<commit_message>
CCD-6594: reject FixedLists CaseTypeID values that are not a case type
The CaseTypeID now changes the identity of the generated field types, so a
typo or the case type name instead of its ID quietly produces list types that
no case field can reference. Fail the import with the offending value instead.

The V12 test definition was using case type names, so its CaseTypeID column
has been corrected to TestAddressBookCase / TestComplexAddressBookCase.

Also report the FixedList reference against FixedList rather than
FixedRadioList when it exceeds the column length, which scoping makes more
likely to be hit.
</commit_message>
<xml_diff>
--- a/excel-importer/src/test/resources/CCD_TestDefinition_V12_FixedList_CaseType.xlsx
+++ b/excel-importer/src/test/resources/CCD_TestDefinition_V12_FixedList_CaseType.xlsx
@@ -16250,7 +16250,7 @@
         <v>72</v>
       </c>
       <c r="D17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E17" s="66" t="s">
         <v>85</v>
@@ -16290,7 +16290,7 @@
         <v>72</v>
       </c>
       <c r="D18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E18" s="66" t="s">
         <v>87</v>
@@ -16330,7 +16330,7 @@
         <v>72</v>
       </c>
       <c r="D19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E19" s="66" t="s">
         <v>89</v>
@@ -16370,7 +16370,7 @@
         <v>72</v>
       </c>
       <c r="D20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E20" s="66" t="s">
         <v>91</v>
@@ -16410,7 +16410,7 @@
         <v>76</v>
       </c>
       <c r="D21" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E21" s="66" t="s">
         <v>93</v>
@@ -16450,7 +16450,7 @@
         <v>76</v>
       </c>
       <c r="D22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E22" s="66" t="s">
         <v>95</v>
@@ -16490,7 +16490,7 @@
         <v>76</v>
       </c>
       <c r="D23" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E23" s="66" t="s">
         <v>97</v>
@@ -16530,7 +16530,7 @@
         <v>258</v>
       </c>
       <c r="D24" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E24" s="66" t="s">
         <v>261</v>
@@ -16570,7 +16570,7 @@
         <v>258</v>
       </c>
       <c r="D25" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E25" s="66" t="s">
         <v>262</v>
@@ -16610,7 +16610,7 @@
         <v>259</v>
       </c>
       <c r="D26" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E26" s="66" t="s">
         <v>261</v>
@@ -16650,7 +16650,7 @@
         <v>259</v>
       </c>
       <c r="D27" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E27" s="66" t="s">
         <v>262</v>
@@ -16690,7 +16690,7 @@
         <v>260</v>
       </c>
       <c r="D28" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E28" s="66" t="s">
         <v>261</v>
@@ -16730,7 +16730,7 @@
         <v>260</v>
       </c>
       <c r="D29" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E29" s="66" t="s">
         <v>262</v>

</xml_diff>